<commit_message>
log-sum-exp in the mixed logit likelihood
</commit_message>
<xml_diff>
--- a/examples/output/MXL_routeChoice.xlsx
+++ b/examples/output/MXL_routeChoice.xlsx
@@ -495,22 +495,22 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>-2.063714382319227</v>
+        <v>-2.063714306733265</v>
       </c>
       <c r="C2">
-        <v>0.13161056748307118</v>
+        <v>0.13161057371092916</v>
       </c>
       <c r="D2">
-        <v>-15.680461088997879</v>
+        <v>-15.680459772677754</v>
       </c>
       <c r="E2">
         <v>0.0</v>
       </c>
       <c r="F2">
-        <v>0.15442872480983205</v>
+        <v>0.15442871415692963</v>
       </c>
       <c r="G2">
-        <v>-13.363539619073743</v>
+        <v>-13.363540051470801</v>
       </c>
       <c r="H2">
         <v>0.0</v>
@@ -521,22 +521,22 @@
         <v>9</v>
       </c>
       <c r="B3">
-        <v>-3.817987309240455</v>
+        <v>-3.8179856567179633</v>
       </c>
       <c r="C3">
-        <v>0.2743073509484465</v>
+        <v>0.27430720325706326</v>
       </c>
       <c r="D3">
-        <v>-13.918647444333383</v>
+        <v>-13.918648914006061</v>
       </c>
       <c r="E3">
         <v>0.0</v>
       </c>
       <c r="F3">
-        <v>0.3138202806980432</v>
+        <v>0.31382003829120975</v>
       </c>
       <c r="G3">
-        <v>-12.16615860755701</v>
+        <v>-12.16616273934381</v>
       </c>
       <c r="H3">
         <v>0.0</v>
@@ -547,22 +547,22 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>-4.370268733702974</v>
+        <v>-4.370268054469075</v>
       </c>
       <c r="C4">
-        <v>0.40919661634317955</v>
+        <v>0.4091964726369675</v>
       </c>
       <c r="D4">
-        <v>-10.680119431969533</v>
+        <v>-10.680121522812602</v>
       </c>
       <c r="E4">
         <v>0.0</v>
       </c>
       <c r="F4">
-        <v>0.5488302915255884</v>
+        <v>0.5488298998683507</v>
       </c>
       <c r="G4">
-        <v>-7.962878144999795</v>
+        <v>-7.962882589883281</v>
       </c>
       <c r="H4">
         <v>1.7763568394002505e-15</v>
@@ -573,22 +573,22 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>-8.106013042125305</v>
+        <v>-8.106013908874315</v>
       </c>
       <c r="C5">
-        <v>0.6230548025335906</v>
+        <v>0.6230548336654801</v>
       </c>
       <c r="D5">
-        <v>-13.010112447834455</v>
+        <v>-13.010113188892227</v>
       </c>
       <c r="E5">
         <v>0.0</v>
       </c>
       <c r="F5">
-        <v>0.8238641288428898</v>
+        <v>0.8238640479992062</v>
       </c>
       <c r="G5">
-        <v>-9.839016845544824</v>
+        <v>-9.83901886307597</v>
       </c>
       <c r="H5">
         <v>0.0</v>
@@ -599,22 +599,22 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>1.280268681972284</v>
+        <v>1.280269259312368</v>
       </c>
       <c r="C6">
-        <v>0.1375362820549591</v>
+        <v>0.13753632027766727</v>
       </c>
       <c r="D6">
-        <v>9.308588707237936</v>
+        <v>9.308590318016922</v>
       </c>
       <c r="E6">
         <v>0.0</v>
       </c>
       <c r="F6">
-        <v>0.16198930293441824</v>
+        <v>0.16198932372514524</v>
       </c>
       <c r="G6">
-        <v>7.903414971114505</v>
+        <v>7.90341752080316</v>
       </c>
       <c r="H6">
         <v>2.6645352591003757e-15</v>
@@ -625,25 +625,25 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>2.4330367607884407</v>
+        <v>2.433035402294796</v>
       </c>
       <c r="C7">
-        <v>0.31293085556526556</v>
+        <v>0.31293078844169964</v>
       </c>
       <c r="D7">
-        <v>7.774997950884396</v>
+        <v>7.77499527742404</v>
       </c>
       <c r="E7">
         <v>7.549516567451064e-15</v>
       </c>
       <c r="F7">
-        <v>0.38709732688878956</v>
+        <v>0.387097243497123</v>
       </c>
       <c r="G7">
-        <v>6.285335991192302</v>
+        <v>6.285333835793328</v>
       </c>
       <c r="H7">
-        <v>3.2714542186340623e-10</v>
+        <v>3.2714986275550473e-10</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -651,22 +651,22 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>3.7247345518949975</v>
+        <v>3.7247339177022374</v>
       </c>
       <c r="C8">
-        <v>0.39600477562977104</v>
+        <v>0.3960046299175703</v>
       </c>
       <c r="D8">
-        <v>9.405781902431627</v>
+        <v>9.405783761865495</v>
       </c>
       <c r="E8">
         <v>0.0</v>
       </c>
       <c r="F8">
-        <v>0.510151949097205</v>
+        <v>0.5101514897143139</v>
       </c>
       <c r="G8">
-        <v>7.301225759279187</v>
+        <v>7.301231090765015</v>
       </c>
       <c r="H8">
         <v>2.851052727237402e-13</v>
@@ -677,25 +677,25 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>3.985404087517425</v>
+        <v>3.9854053303985033</v>
       </c>
       <c r="C9">
-        <v>0.6862289393030652</v>
+        <v>0.6862288102223716</v>
       </c>
       <c r="D9">
-        <v>5.807688745340593</v>
+        <v>5.807691648951663</v>
       </c>
       <c r="E9">
-        <v>6.33411278982976e-9</v>
+        <v>6.334003099794927e-9</v>
       </c>
       <c r="F9">
-        <v>0.770269306634805</v>
+        <v>0.7702690432387344</v>
       </c>
       <c r="G9">
-        <v>5.174039849684623</v>
+        <v>5.1740432325323</v>
       </c>
       <c r="H9">
-        <v>2.2908593200199334e-7</v>
+        <v>2.290817822103719e-7</v>
       </c>
     </row>
   </sheetData>
@@ -713,7 +713,7 @@
         <v>16</v>
       </c>
       <c r="B1">
-        <v>-1471.0018587449435</v>
+        <v>-1471.001858744893</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -729,7 +729,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -753,7 +753,7 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>2.9844770431518555</v>
+        <v>2.8855741024017334</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -777,7 +777,7 @@
         <v>25</v>
       </c>
       <c r="B9">
-        <v>2958.003717489887</v>
+        <v>2958.003717489786</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -785,7 +785,7 @@
         <v>26</v>
       </c>
       <c r="B10">
-        <v>3007.269556825563</v>
+        <v>3007.269556825462</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -793,7 +793,7 @@
         <v>27</v>
       </c>
       <c r="B11">
-        <v>0.39226601181277154</v>
+        <v>0.3922660118127924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>